<commit_message>
Update two xlsx files
</commit_message>
<xml_diff>
--- a/OG0005/OG0005_ReadingQuiz.xlsx
+++ b/OG0005/OG0005_ReadingQuiz.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IM_1075\Documents\GitHub\reading-quiz\OG0005\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{629F05A4-BBF1-4468-BD85-FDABB9381A53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32C93C84-6185-461F-9B6F-3732644BFDA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="43080" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1149,19 +1149,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1172,12 +1166,6 @@
       <i/>
       <sz val="9"/>
       <color rgb="FF6B7280"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF5B21B6"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1253,7 +1241,7 @@
       <charset val="129"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1262,37 +1250,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF5F3FF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF7C3AED"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFEDE9FE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFECFDF5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFEDD5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFEF2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -1345,8 +1303,13 @@
         <fgColor rgb="FFFFEECC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -1426,165 +1389,215 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1902,263 +1915,263 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
-      <c r="J1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
+      <c r="J1" s="30"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="9" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="9" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="9" t="s">
+      <c r="J2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="I3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="10" t="s">
+      <c r="J3" s="3" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="10" t="s">
+      <c r="H4" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="I4" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="J4" s="10" t="s">
+      <c r="J4" s="3" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="I5" s="10" t="s">
+      <c r="I5" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="J5" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="J6" s="10" t="s">
+      <c r="J6" s="3" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="J7" s="10" t="s">
+      <c r="J7" s="3" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="J8" s="10" t="s">
+      <c r="J8" s="3" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.6">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="31" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
-      <c r="J10" s="31"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A10:J10"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -2180,468 +2193,468 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
     </row>
     <row r="2" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
-      <c r="J2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
     </row>
     <row r="3" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="38" t="s">
         <v>62</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
     </row>
     <row r="4" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="39" t="s">
+      <c r="A4" s="40" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-      <c r="J4" s="31"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+      <c r="J4" s="32"/>
     </row>
     <row r="5" spans="1:10" ht="22.05" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="31"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="31"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="31"/>
+      <c r="B5" s="32"/>
+      <c r="C5" s="32"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="32"/>
+      <c r="J5" s="32"/>
     </row>
     <row r="6" spans="1:10" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6"/>
     <row r="7" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="35" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="35"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
-      <c r="E7" s="35"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="35"/>
-      <c r="H7" s="35"/>
-      <c r="I7" s="35"/>
-      <c r="J7" s="35"/>
+      <c r="B7" s="36"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="36"/>
+      <c r="H7" s="36"/>
+      <c r="I7" s="36"/>
+      <c r="J7" s="36"/>
     </row>
     <row r="8" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="B8" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="9" t="s">
+      <c r="D8" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="9" t="s">
+      <c r="E8" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="2" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="6">
         <v>1</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="6">
         <v>2.5</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="6">
         <f>D9/SUM($D$9:$D$13)*100</f>
         <v>26.315789473684209</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="14" t="s">
+      <c r="A10" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="8">
         <v>2</v>
       </c>
-      <c r="C10" s="14" t="s">
+      <c r="C10" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="D10" s="15">
+      <c r="D10" s="8">
         <v>1.5</v>
       </c>
-      <c r="E10" s="14" t="s">
+      <c r="E10" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="8">
         <f>D10/SUM($D$9:$D$13)*100</f>
         <v>15.789473684210526</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B11" s="15">
+      <c r="B11" s="8">
         <v>3</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D11" s="15">
+      <c r="D11" s="8">
         <v>1.5</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="8">
         <f>D11/SUM($D$9:$D$13)*100</f>
         <v>15.789473684210526</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="8">
         <v>4</v>
       </c>
-      <c r="C12" s="14" t="s">
+      <c r="C12" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="8">
         <v>1.5</v>
       </c>
-      <c r="E12" s="14" t="s">
+      <c r="E12" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="8">
         <f>D12/SUM($D$9:$D$13)*100</f>
         <v>15.789473684210526</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="B13" s="13">
+      <c r="B13" s="6">
         <v>5</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="6">
         <v>2.5</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="E13" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="F13" s="13">
+      <c r="F13" s="6">
         <f>D13/SUM($D$9:$D$13)*100</f>
         <v>26.315789473684209</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.6">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="17"/>
-      <c r="C14" s="17"/>
-      <c r="D14" s="16">
+      <c r="B14" s="10"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="9">
         <f>SUM(D9:D13)</f>
         <v>9.5</v>
       </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="16">
+      <c r="E14" s="10"/>
+      <c r="F14" s="9">
         <f>SUM(F9:F13)</f>
         <v>99.999999999999986</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="38" t="s">
+      <c r="A16" s="39" t="s">
         <v>88</v>
       </c>
-      <c r="B16" s="31"/>
-      <c r="C16" s="31"/>
-      <c r="D16" s="31"/>
-      <c r="E16" s="31"/>
-      <c r="F16" s="31"/>
-      <c r="G16" s="31"/>
-      <c r="H16" s="31"/>
-      <c r="I16" s="31"/>
-      <c r="J16" s="31"/>
+      <c r="B16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="32"/>
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="32"/>
+      <c r="I16" s="32"/>
+      <c r="J16" s="32"/>
     </row>
     <row r="17" spans="1:10" ht="39.4" x14ac:dyDescent="0.6">
-      <c r="A17" s="18" t="s">
+      <c r="A17" s="11" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="B17" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="9" t="s">
+      <c r="D17" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="2" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A18" s="19" t="s">
+      <c r="A18" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="13">
         <v>26.3</v>
       </c>
-      <c r="C18" s="21">
+      <c r="C18" s="14">
         <v>13.2</v>
       </c>
-      <c r="D18" s="22">
+      <c r="D18" s="15">
         <v>0</v>
       </c>
-      <c r="E18" s="22">
+      <c r="E18" s="15">
         <v>0</v>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A19" s="19" t="s">
+      <c r="A19" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B19" s="21">
+      <c r="B19" s="14">
         <v>7.9</v>
       </c>
-      <c r="C19" s="20">
+      <c r="C19" s="13">
         <v>15.8</v>
       </c>
-      <c r="D19" s="21">
+      <c r="D19" s="14">
         <v>7.9</v>
       </c>
-      <c r="E19" s="22">
+      <c r="E19" s="15">
         <v>0</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="19" t="s">
+      <c r="A20" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="15">
         <v>0</v>
       </c>
-      <c r="C20" s="21">
+      <c r="C20" s="14">
         <v>7.9</v>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="13">
         <v>15.8</v>
       </c>
-      <c r="E20" s="21">
+      <c r="E20" s="14">
         <v>7.9</v>
       </c>
-      <c r="F20" s="22">
+      <c r="F20" s="15">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A21" s="19" t="s">
+      <c r="A21" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="15">
         <v>0</v>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="15">
         <v>0</v>
       </c>
-      <c r="D21" s="21">
+      <c r="D21" s="14">
         <v>7.9</v>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="13">
         <v>15.8</v>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="14">
         <v>7.9</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="B22" s="22">
+      <c r="B22" s="15">
         <v>0</v>
       </c>
-      <c r="C22" s="22">
+      <c r="C22" s="15">
         <v>0</v>
       </c>
-      <c r="D22" s="22">
+      <c r="D22" s="15">
         <v>0</v>
       </c>
-      <c r="E22" s="21">
+      <c r="E22" s="14">
         <v>13.2</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="13">
         <v>26.3</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6"/>
     <row r="24" spans="1:10" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A24" s="36" t="s">
+      <c r="A24" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="B24" s="29"/>
-      <c r="C24" s="29"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
-      <c r="I24" s="31"/>
-      <c r="J24" s="31"/>
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="32"/>
+      <c r="F24" s="32"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="32"/>
+      <c r="I24" s="32"/>
+      <c r="J24" s="32"/>
     </row>
     <row r="25" spans="1:10" ht="47.25" x14ac:dyDescent="0.6">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="B25" s="23" t="s">
+      <c r="B25" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="D25" s="23" t="s">
+      <c r="D25" s="16" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C26" s="24">
+      <c r="C26" s="17">
         <v>100</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="3" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="52.5" x14ac:dyDescent="0.6">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C27" s="25">
+      <c r="C27" s="18">
         <v>79</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="3" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="39.4" x14ac:dyDescent="0.6">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="C28" s="26">
+      <c r="C28" s="19">
         <v>53</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" s="3" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="39.4" x14ac:dyDescent="0.6">
-      <c r="A29" s="10" t="s">
+      <c r="A29" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C29" s="26">
+      <c r="C29" s="19">
         <v>28</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" s="3" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.6">
-      <c r="A30" s="27"/>
-      <c r="B30" s="27"/>
-      <c r="D30" s="27"/>
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+      <c r="D30" s="20"/>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.6">
-      <c r="A31" s="30" t="s">
+      <c r="A31" s="31" t="s">
         <v>111</v>
       </c>
-      <c r="B31" s="31"/>
-      <c r="C31" s="31"/>
-      <c r="D31" s="31"/>
-      <c r="E31" s="31"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="31"/>
-      <c r="H31" s="31"/>
-      <c r="I31" s="31"/>
-      <c r="J31" s="31"/>
+      <c r="B31" s="32"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="32"/>
+      <c r="E31" s="32"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="32"/>
+      <c r="H31" s="32"/>
+      <c r="I31" s="32"/>
+      <c r="J31" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2655,7 +2668,7 @@
     <mergeCell ref="A4:J4"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2675,225 +2688,225 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="49" t="s">
+      <c r="A1" s="43" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-      <c r="E1" s="29"/>
-      <c r="F1" s="29"/>
-      <c r="G1" s="29"/>
-      <c r="H1" s="29"/>
-      <c r="I1" s="29"/>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30"/>
+      <c r="H1" s="30"/>
+      <c r="I1" s="30"/>
     </row>
     <row r="2" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="42" t="s">
         <v>113</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
     </row>
     <row r="3" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="51" t="s">
+      <c r="A3" s="44" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29"/>
-      <c r="I3" s="29"/>
-    </row>
-    <row r="4" spans="1:9" s="8" customFormat="1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="52"/>
-      <c r="B4" s="52"/>
-      <c r="C4" s="52"/>
-      <c r="D4" s="52"/>
-      <c r="E4" s="52"/>
-      <c r="F4" s="52"/>
-      <c r="G4" s="52"/>
-      <c r="H4" s="52"/>
-      <c r="I4" s="52"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+      <c r="I3" s="30"/>
+    </row>
+    <row r="4" spans="1:9" s="1" customFormat="1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="25"/>
+      <c r="H4" s="25"/>
+      <c r="I4" s="25"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="45" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="42"/>
-      <c r="I5" s="43"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="46"/>
+      <c r="I5" s="47"/>
     </row>
     <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="F6" s="11" t="s">
+      <c r="F6" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="E7" s="25">
+      <c r="E7" s="18">
         <v>25</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="5" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D8" s="24" t="s">
+      <c r="D8" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="E8" s="24">
+      <c r="E8" s="17">
         <v>100</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="3" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="5">
         <v>15</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="3" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="19">
         <v>5</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="H10" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="I10" s="10" t="s">
+      <c r="I10" s="3" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="31" t="s">
         <v>144</v>
       </c>
-      <c r="B11" s="31"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31"/>
-      <c r="F11" s="31"/>
-      <c r="G11" s="31"/>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31"/>
+      <c r="B11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="32"/>
+      <c r="I11" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2903,7 +2916,7 @@
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A5:I5"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2921,414 +2934,414 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
     </row>
     <row r="2" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="40" t="s">
+      <c r="A2" s="41" t="s">
         <v>146</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
-      <c r="D2" s="31"/>
-      <c r="E2" s="31"/>
-      <c r="F2" s="31"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="31"/>
-      <c r="I2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
     </row>
     <row r="3" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A3" s="37" t="s">
+      <c r="A3" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
     </row>
     <row r="4" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="34" t="s">
         <v>148</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
-      <c r="I4" s="31"/>
-    </row>
-    <row r="5" spans="1:9" s="8" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.6"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="32"/>
+      <c r="I4" s="32"/>
+    </row>
+    <row r="5" spans="1:9" s="1" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.6"/>
     <row r="6" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="37" t="s">
         <v>149</v>
       </c>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="31"/>
-      <c r="I6" s="31"/>
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32"/>
     </row>
     <row r="7" spans="1:9" ht="31.5" x14ac:dyDescent="0.6">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="C7" s="4" t="s">
         <v>151</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="F7" s="11" t="s">
+      <c r="F7" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" s="4" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="B8" s="56">
+      <c r="B8" s="28">
         <v>1</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="D8" s="56">
+      <c r="D8" s="28">
         <v>1.5</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="8">
         <f t="shared" ref="F8:F14" si="0">D8/SUM($D$8:$D$14)*100</f>
         <v>12</v>
       </c>
-      <c r="G8" s="56">
+      <c r="G8" s="28">
         <f>F8</f>
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="B9" s="56">
+      <c r="B9" s="28">
         <v>2</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="D9" s="56">
+      <c r="D9" s="28">
         <v>2.5</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="F9" s="15">
+      <c r="F9" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="G9" s="56">
+      <c r="G9" s="28">
         <f>F8+F9</f>
         <v>32</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="B10" s="56">
+      <c r="B10" s="28">
         <v>3</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="D10" s="56">
+      <c r="D10" s="28">
         <v>1</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F10" s="15">
+      <c r="F10" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="G10" s="56">
+      <c r="G10" s="28">
         <f>F8+F9+F10</f>
         <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="5" t="s">
         <v>163</v>
       </c>
-      <c r="B11" s="56">
+      <c r="B11" s="28">
         <v>4</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="D11" s="56">
+      <c r="D11" s="28">
         <v>1.5</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="F11" s="15">
+      <c r="F11" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="G11" s="56">
+      <c r="G11" s="28">
         <f>F8+F9+F10+F11</f>
         <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="B12" s="56">
+      <c r="B12" s="28">
         <v>5</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D12" s="56">
+      <c r="D12" s="28">
         <v>2.5</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="F12" s="15">
+      <c r="F12" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="G12" s="56">
+      <c r="G12" s="28">
         <f>F8+F9+F10+F11+F12</f>
         <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="5" t="s">
         <v>169</v>
       </c>
-      <c r="B13" s="56">
+      <c r="B13" s="28">
         <v>6</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="D13" s="56">
+      <c r="D13" s="28">
         <v>1.5</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="F13" s="15">
+      <c r="F13" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="G13" s="56">
+      <c r="G13" s="28">
         <f>F8+F9+F10+F11+F12+F13</f>
         <v>84</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="B14" s="56">
+      <c r="B14" s="28">
         <v>7</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="D14" s="56">
+      <c r="D14" s="28">
         <v>2</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="F14" s="15">
+      <c r="F14" s="8">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="G14" s="56">
+      <c r="G14" s="28">
         <f>SUM(F8:F14)</f>
         <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="16">
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="9">
         <f>SUM(D8:D14)</f>
         <v>12.5</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="16">
+      <c r="E15" s="10"/>
+      <c r="F15" s="9">
         <f>SUM(F8:F14)</f>
         <v>100</v>
       </c>
-      <c r="G15" s="16" t="s">
+      <c r="G15" s="9" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="16" spans="1:9" s="8" customFormat="1" x14ac:dyDescent="0.6">
-      <c r="A16" s="55"/>
+    <row r="16" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A16" s="27"/>
     </row>
     <row r="17" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A17" s="36" t="s">
+      <c r="A17" s="37" t="s">
         <v>176</v>
       </c>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
-      <c r="D17" s="29"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="29"/>
-      <c r="G17" s="29"/>
-      <c r="H17" s="31"/>
-      <c r="I17" s="31"/>
+      <c r="B17" s="30"/>
+      <c r="C17" s="30"/>
+      <c r="D17" s="30"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="30"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="32"/>
+      <c r="I17" s="32"/>
     </row>
     <row r="18" spans="1:9" ht="31.5" x14ac:dyDescent="0.6">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="16" t="s">
         <v>177</v>
       </c>
-      <c r="B18" s="23" t="s">
+      <c r="B18" s="16" t="s">
         <v>178</v>
       </c>
-      <c r="C18" s="23" t="s">
+      <c r="C18" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="D18" s="23" t="s">
+      <c r="D18" s="16" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="19" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="C19" s="24">
+      <c r="C19" s="17">
         <v>100</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="3" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="C20" s="25">
+      <c r="C20" s="18">
         <v>84</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="3" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="21" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="C21" s="25">
+      <c r="C21" s="18">
         <v>52</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="3" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="22" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="3" t="s">
         <v>187</v>
       </c>
-      <c r="C22" s="25">
+      <c r="C22" s="18">
         <v>68</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="3" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C23" s="26">
+      <c r="C23" s="19">
         <v>28</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="3" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="3" t="s">
         <v>193</v>
       </c>
-      <c r="C24" s="26">
+      <c r="C24" s="19">
         <v>0</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="3" t="s">
         <v>194</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="31" t="s">
         <v>195</v>
       </c>
-      <c r="B25" s="31"/>
-      <c r="C25" s="31"/>
-      <c r="D25" s="31"/>
-      <c r="E25" s="31"/>
-      <c r="F25" s="31"/>
-      <c r="G25" s="31"/>
-      <c r="H25" s="31"/>
-      <c r="I25" s="31"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3340,7 +3353,7 @@
     <mergeCell ref="A3:I3"/>
     <mergeCell ref="A4:I4"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3360,211 +3373,211 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>196</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
     </row>
     <row r="2" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A2" s="50" t="s">
+      <c r="A2" s="42" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="29"/>
-    </row>
-    <row r="3" spans="1:9" s="8" customFormat="1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="B3" s="52"/>
-      <c r="C3" s="52"/>
-      <c r="D3" s="52"/>
-      <c r="E3" s="52"/>
-      <c r="F3" s="52"/>
-      <c r="G3" s="52"/>
-      <c r="H3" s="52"/>
-      <c r="I3" s="52"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+    </row>
+    <row r="3" spans="1:9" s="1" customFormat="1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A4" s="46" t="s">
+      <c r="A4" s="48" t="s">
         <v>198</v>
       </c>
-      <c r="B4" s="42"/>
-      <c r="C4" s="42"/>
-      <c r="D4" s="42"/>
-      <c r="E4" s="42"/>
-      <c r="F4" s="42"/>
-      <c r="G4" s="42"/>
-      <c r="H4" s="42"/>
-      <c r="I4" s="43"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="47"/>
     </row>
     <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="C5" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="F5" s="11" t="s">
+      <c r="F5" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="G5" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="H5" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="I5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="18" t="s">
         <v>122</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="C6" s="25" t="s">
+      <c r="C6" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="18">
         <v>50</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="3" t="s">
         <v>203</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="I6" s="10" t="s">
+      <c r="I6" s="3" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="D7" s="24">
+      <c r="D7" s="17">
         <v>100</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="3" t="s">
         <v>209</v>
       </c>
-      <c r="H7" s="10" t="s">
+      <c r="H7" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A8" s="53" t="s">
+      <c r="A8" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="C8" s="53" t="s">
+      <c r="C8" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D8" s="53">
+      <c r="D8" s="26">
         <v>0</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="H8" s="10" t="s">
+      <c r="H8" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="I8" s="10" t="s">
+      <c r="I8" s="3" t="s">
         <v>206</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A9" s="53" t="s">
+      <c r="A9" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="C9" s="53" t="s">
+      <c r="C9" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D9" s="53">
+      <c r="D9" s="26">
         <v>20</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="I9" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="31" t="s">
         <v>220</v>
       </c>
-      <c r="B10" s="31"/>
-      <c r="C10" s="31"/>
-      <c r="D10" s="31"/>
-      <c r="E10" s="31"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="31"/>
-      <c r="H10" s="31"/>
-      <c r="I10" s="31"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -3573,822 +3586,835 @@
     <mergeCell ref="A10:I10"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="7" width="46" customWidth="1"/>
-    <col min="8" max="8" width="50" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="11.9375" customWidth="1"/>
+    <col min="4" max="5" width="20" customWidth="1"/>
+    <col min="6" max="7" width="24" customWidth="1"/>
+    <col min="8" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>221</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A2" s="41" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+    </row>
+    <row r="2" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A2" s="42" t="s">
         <v>222</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="43"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A3" s="44" t="s">
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+    </row>
+    <row r="3" spans="1:9" s="21" customFormat="1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.6">
+      <c r="A4" s="49" t="s">
         <v>223</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="43"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A4" s="1" t="s">
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
+      <c r="H4" s="46"/>
+      <c r="I4" s="47"/>
+    </row>
+    <row r="5" spans="1:9" ht="31.5" x14ac:dyDescent="0.6">
+      <c r="A5" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D5" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E5" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F5" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G5" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H5" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I5" s="22" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A5" s="4" t="s">
+    <row r="6" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A6" s="17" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C6" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D6" s="17">
         <v>100</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E6" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F6" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H6" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A6" s="3" t="s">
+    <row r="7" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="19" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B7" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C7" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D7" s="19">
         <v>0</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>227</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H7" s="3" t="s">
         <v>229</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="I7" s="3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A7" s="2" t="s">
+    <row r="8" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A8" s="18" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C8" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D8" s="18">
         <v>20</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>231</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G8" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H8" s="3" t="s">
         <v>234</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A8" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="D8" s="3">
-        <v>10</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>237</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>238</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>239</v>
       </c>
       <c r="I8" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A9" s="30" t="s">
+    <row r="9" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A9" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="26">
+        <v>10</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.6">
+      <c r="A10" s="31" t="s">
         <v>240</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="A10:I10"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="8" width="52" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="5" width="20" customWidth="1"/>
+    <col min="6" max="8" width="24" customWidth="1"/>
     <col min="9" max="9" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>241</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A2" s="41" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+    </row>
+    <row r="2" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A2" s="54" t="s">
         <v>242</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="I2" s="43"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A3" s="44" t="s">
+      <c r="B2" s="55"/>
+      <c r="C2" s="55"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
+      <c r="H2" s="55"/>
+      <c r="I2" s="56"/>
+    </row>
+    <row r="3" spans="1:9" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A3" s="57" t="s">
         <v>243</v>
       </c>
-      <c r="B3" s="42"/>
-      <c r="C3" s="42"/>
-      <c r="D3" s="42"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="42"/>
-      <c r="G3" s="42"/>
-      <c r="H3" s="42"/>
-      <c r="I3" s="43"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A4" s="1" t="s">
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="58"/>
+      <c r="G3" s="58"/>
+      <c r="H3" s="58"/>
+      <c r="I3" s="59"/>
+    </row>
+    <row r="4" spans="1:9" s="21" customFormat="1" ht="16.899999999999999" customHeight="1" x14ac:dyDescent="0.6"/>
+    <row r="5" spans="1:9" ht="31.5" x14ac:dyDescent="0.6">
+      <c r="A5" s="22" t="s">
         <v>116</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B5" s="22" t="s">
         <v>199</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D5" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E5" s="22" t="s">
         <v>68</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F5" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G5" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="H5" s="22" t="s">
         <v>121</v>
       </c>
-      <c r="I4" s="1" t="s">
+      <c r="I5" s="22" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A5" s="2" t="s">
+    <row r="6" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A6" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C6" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D6" s="26">
         <v>10</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E6" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F6" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G6" s="3" t="s">
         <v>247</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H6" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="I6" s="3" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A6" s="4" t="s">
+    <row r="7" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C7" s="17" t="s">
         <v>130</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D7" s="17">
         <v>100</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E7" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="F7" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H7" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I7" s="3" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A7" s="2" t="s">
+    <row r="8" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A8" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C8" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D8" s="26">
         <v>20</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E8" s="3" t="s">
         <v>253</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G8" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H8" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="I8" s="3" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A8" s="3" t="s">
+    <row r="9" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A9" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>257</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C9" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D9" s="26">
         <v>0</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="I8" s="3" t="s">
+      <c r="I9" s="3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.6">
-      <c r="A9" s="30" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.6">
+      <c r="A10" s="31" t="s">
         <v>262</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
-      <c r="I9" s="31"/>
+      <c r="B10" s="32"/>
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A3:I3"/>
-    <mergeCell ref="A9:I9"/>
+    <mergeCell ref="A10:I10"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="16.899999999999999" x14ac:dyDescent="0.6"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="24" customWidth="1"/>
-    <col min="7" max="7" width="36" customWidth="1"/>
+    <col min="1" max="1" width="10" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="5" width="18" customWidth="1"/>
+    <col min="6" max="7" width="28" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>263</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A2" s="45" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+    </row>
+    <row r="2" spans="1:7" s="21" customFormat="1" ht="26" customHeight="1" x14ac:dyDescent="0.6"/>
+    <row r="3" spans="1:7" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A3" s="37" t="s">
         <v>264</v>
       </c>
-      <c r="B2" s="42"/>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="E2" s="42"/>
-      <c r="F2" s="42"/>
-      <c r="G2" s="43"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A3" s="1" t="s">
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.6">
+      <c r="A4" s="16" t="s">
         <v>265</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B4" s="16" t="s">
         <v>266</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C4" s="16" t="s">
         <v>267</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D4" s="16" t="s">
         <v>268</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E4" s="16" t="s">
         <v>269</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F4" s="16" t="s">
         <v>270</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G4" s="16" t="s">
         <v>271</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A4" s="4" t="s">
+    <row r="5" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A5" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>275</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F5" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A5" s="5" t="s">
+    <row r="6" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A6" s="3" t="s">
         <v>279</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B6" s="24" t="s">
         <v>280</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C6" s="3" t="s">
         <v>281</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D6" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E6" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F6" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G6" s="3" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A6" s="6" t="s">
+    <row r="7" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A7" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B7" s="60" t="s">
         <v>287</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C7" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D7" s="3" t="s">
         <v>289</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E7" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F7" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G7" s="3" t="s">
         <v>292</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A7" s="7" t="s">
+    <row r="8" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A8" s="3" t="s">
         <v>293</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B8" s="19" t="s">
         <v>294</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C8" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D8" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E8" s="3" t="s">
         <v>297</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F8" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G8" s="3" t="s">
         <v>299</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A8" s="45" t="s">
+    <row r="9" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.6"/>
+    <row r="10" spans="1:7" s="21" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A10" s="37" t="s">
         <v>300</v>
       </c>
-      <c r="B8" s="42"/>
-      <c r="C8" s="42"/>
-      <c r="D8" s="42"/>
-      <c r="E8" s="42"/>
-      <c r="F8" s="42"/>
-      <c r="G8" s="43"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A9" s="1" t="s">
+      <c r="B10" s="30"/>
+      <c r="C10" s="30"/>
+      <c r="D10" s="30"/>
+      <c r="E10" s="30"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="30"/>
+    </row>
+    <row r="11" spans="1:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A11" s="16" t="s">
         <v>301</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B11" s="16" t="s">
         <v>302</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C11" s="16" t="s">
         <v>303</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D11" s="16" t="s">
         <v>304</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E11" s="16" t="s">
         <v>305</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A10" s="3" t="s">
+    <row r="12" spans="1:7" ht="39.4" x14ac:dyDescent="0.6">
+      <c r="A12" s="24" t="s">
         <v>306</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>307</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>308</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>309</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A12" s="3" t="s">
-        <v>314</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>315</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>316</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>309</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A13" s="2" t="s">
-        <v>318</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>319</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>321</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A14" s="3" t="s">
-        <v>323</v>
+        <v>310</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="39.4" x14ac:dyDescent="0.6">
+      <c r="A13" s="24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="39.4" x14ac:dyDescent="0.6">
+      <c r="A14" s="24" t="s">
+        <v>314</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>309</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="39.4" x14ac:dyDescent="0.6">
+      <c r="A15" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="39.4" x14ac:dyDescent="0.6">
+      <c r="A16" s="24" t="s">
+        <v>323</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>325</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>326</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A15" s="2" t="s">
+    <row r="17" spans="1:7" ht="26.25" x14ac:dyDescent="0.6">
+      <c r="A17" s="24" t="s">
         <v>327</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C17" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D17" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E17" s="3" t="s">
         <v>330</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="26.25" x14ac:dyDescent="0.6">
-      <c r="A16" s="3" t="s">
+    <row r="18" spans="1:7" ht="39.4" x14ac:dyDescent="0.6">
+      <c r="A18" s="24" t="s">
         <v>331</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B18" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A17" s="45" t="s">
+    <row r="19" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.6"/>
+    <row r="20" spans="1:7" s="21" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A20" s="37" t="s">
         <v>334</v>
       </c>
-      <c r="B17" s="42"/>
-      <c r="C17" s="42"/>
-      <c r="D17" s="42"/>
-      <c r="E17" s="42"/>
-      <c r="F17" s="42"/>
-      <c r="G17" s="43"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A18" s="47" t="s">
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="30"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="30"/>
+      <c r="G20" s="30"/>
+    </row>
+    <row r="21" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A21" s="53" t="s">
         <v>335</v>
       </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="31"/>
-      <c r="E18" s="31"/>
-      <c r="F18" s="31"/>
-      <c r="G18" s="31"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A19" s="47" t="s">
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
+      <c r="D21" s="30"/>
+      <c r="E21" s="30"/>
+      <c r="F21" s="30"/>
+      <c r="G21" s="30"/>
+    </row>
+    <row r="22" spans="1:7" ht="28.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A22" s="61" t="s">
         <v>336</v>
       </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
-      <c r="D19" s="31"/>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="31"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A20" s="45" t="s">
+      <c r="B22" s="30"/>
+      <c r="C22" s="30"/>
+      <c r="D22" s="30"/>
+      <c r="E22" s="30"/>
+      <c r="F22" s="30"/>
+      <c r="G22" s="30"/>
+    </row>
+    <row r="23" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.6">
+      <c r="A23" s="23"/>
+    </row>
+    <row r="24" spans="1:7" s="21" customFormat="1" ht="22.15" customHeight="1" x14ac:dyDescent="0.6">
+      <c r="A24" s="37" t="s">
         <v>337</v>
       </c>
-      <c r="B20" s="42"/>
-      <c r="C20" s="42"/>
-      <c r="D20" s="42"/>
-      <c r="E20" s="42"/>
-      <c r="F20" s="42"/>
-      <c r="G20" s="43"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.6">
-      <c r="A21" s="47" t="s">
+      <c r="B24" s="30"/>
+      <c r="C24" s="30"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="30"/>
+      <c r="F24" s="30"/>
+      <c r="G24" s="30"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.6">
+      <c r="A25" s="50" t="s">
         <v>338</v>
       </c>
-      <c r="B21" s="31"/>
-      <c r="C21" s="31"/>
-      <c r="D21" s="31"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
+      <c r="B25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="32"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A21:G21"/>
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A22:G22"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4407,71 +4433,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="26" customHeight="1" x14ac:dyDescent="0.6">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="52" t="s">
         <v>339</v>
       </c>
-      <c r="B1" s="54"/>
-      <c r="C1" s="54"/>
-      <c r="D1" s="54"/>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A2" s="1" t="s">
+      <c r="B1" s="52"/>
+      <c r="C1" s="52"/>
+      <c r="D1" s="52"/>
+      <c r="E1" s="52"/>
+      <c r="F1" s="52"/>
+      <c r="G1" s="52"/>
+      <c r="H1" s="52"/>
+    </row>
+    <row r="2" spans="1:8" ht="31.5" x14ac:dyDescent="0.6">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="22" t="s">
         <v>340</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="22" t="s">
         <v>341</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="22" t="s">
         <v>342</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="22" t="s">
         <v>343</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="22" t="s">
         <v>344</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="22" t="s">
         <v>345</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="22" t="s">
         <v>346</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A3" s="2" t="s">
+    <row r="3" spans="1:8" ht="39.4" x14ac:dyDescent="0.6">
+      <c r="A3" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="3" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:8" ht="26.25" x14ac:dyDescent="0.6">
+      <c r="A4" s="24" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -4496,34 +4522,34 @@
         <v>356</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A5" s="2" t="s">
+    <row r="5" spans="1:8" ht="26.25" x14ac:dyDescent="0.6">
+      <c r="A5" s="24" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>357</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="3" t="s">
         <v>352</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:8" ht="26.25" x14ac:dyDescent="0.6">
+      <c r="A6" s="24" t="s">
         <v>39</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -4548,34 +4574,34 @@
         <v>361</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:8" ht="26.25" x14ac:dyDescent="0.6">
+      <c r="A7" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>347</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" s="3" t="s">
         <v>355</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="3" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:8" ht="26.25" x14ac:dyDescent="0.6">
+      <c r="A8" s="24" t="s">
         <v>53</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -4601,23 +4627,23 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.6">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="51" t="s">
         <v>366</v>
       </c>
-      <c r="B9" s="31"/>
-      <c r="C9" s="31"/>
-      <c r="D9" s="31"/>
-      <c r="E9" s="31"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="31"/>
-      <c r="H9" s="31"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32"/>
+      <c r="H9" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <phoneticPr fontId="7" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>